<commit_message>
fixed colors && work on filters
</commit_message>
<xml_diff>
--- a/Модель покрытия fix.xlsx
+++ b/Модель покрытия fix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mydrive.effem.com/personal/mikhail_gorbunov_effem_com/Documents/Desktop/SPM/Org structure/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\world\Desktop\MARSIntMap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2675056C-6F82-48D2-ACF7-AD089C63B9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DFF98D-8EB9-4A39-96C8-5E6F3DC90017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="8148" yWindow="8148" windowWidth="2388" windowHeight="564" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Исходник" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -194,7 +197,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="297">
   <si>
     <t>District</t>
   </si>
@@ -1091,7 +1094,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1591,7 +1594,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1870,7 +1873,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
@@ -1885,7 +1888,7 @@
     <col min="21" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="43.15">
+    <row r="1" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1947,7 +1950,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -1989,7 +1992,7 @@
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
@@ -2027,7 +2030,7 @@
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
     </row>
-    <row r="4" spans="1:21" ht="28.9">
+    <row r="4" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -2064,7 +2067,7 @@
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -2095,7 +2098,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -2135,7 +2138,7 @@
       </c>
       <c r="R6" s="4"/>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -2172,7 +2175,7 @@
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -2206,7 +2209,7 @@
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
@@ -2234,12 +2237,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -2258,10 +2261,10 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:21">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2269,7 +2272,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18"/>
     </row>
   </sheetData>
@@ -2281,7 +2284,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62F99B76-7CBC-45E3-87BE-CFF232B038A4}">
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
@@ -2296,7 +2299,7 @@
     <col min="28" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="15" thickBot="1">
+    <row r="1" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>45</v>
       </c>
@@ -2324,7 +2327,7 @@
       <c r="Z1" s="51"/>
       <c r="AA1" s="52"/>
     </row>
-    <row r="2" spans="1:28" s="8" customFormat="1" ht="43.9" thickBot="1">
+    <row r="2" spans="1:28" s="8" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I2" s="53" t="s">
         <v>48</v>
       </c>
@@ -2365,7 +2368,7 @@
       <c r="Z2" s="12"/>
       <c r="AA2" s="13"/>
     </row>
-    <row r="3" spans="1:28" s="21" customFormat="1" ht="58.15" thickBot="1">
+    <row r="3" spans="1:28" s="21" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>0</v>
       </c>
@@ -2448,7 +2451,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>20</v>
       </c>
@@ -2501,7 +2504,7 @@
       <c r="Z4" s="28"/>
       <c r="AA4" s="29"/>
     </row>
-    <row r="5" spans="1:28" ht="28.9">
+    <row r="5" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
         <v>20</v>
       </c>
@@ -2548,7 +2551,7 @@
       <c r="Z5" s="36"/>
       <c r="AA5" s="38"/>
     </row>
-    <row r="6" spans="1:28" ht="28.9">
+    <row r="6" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
         <v>20</v>
       </c>
@@ -2593,7 +2596,7 @@
       <c r="Z6" s="36"/>
       <c r="AA6" s="38"/>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="s">
         <v>20</v>
       </c>
@@ -2651,7 +2654,7 @@
       <c r="AA7" s="32"/>
       <c r="AB7"/>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="s">
         <v>35</v>
       </c>
@@ -2704,7 +2707,7 @@
       <c r="Z8" s="30"/>
       <c r="AA8" s="32"/>
     </row>
-    <row r="9" spans="1:28" ht="28.9">
+    <row r="9" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="s">
         <v>35</v>
       </c>
@@ -2751,7 +2754,7 @@
       <c r="Z9" s="36"/>
       <c r="AA9" s="38"/>
     </row>
-    <row r="10" spans="1:28" ht="28.9">
+    <row r="10" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="s">
         <v>35</v>
       </c>
@@ -2796,7 +2799,7 @@
       <c r="Z10" s="36"/>
       <c r="AA10" s="38"/>
     </row>
-    <row r="11" spans="1:28" ht="15" thickBot="1">
+    <row r="11" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="42" t="s">
         <v>35</v>
       </c>
@@ -2853,32 +2856,32 @@
       <c r="Z11" s="42"/>
       <c r="AA11" s="44"/>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:28">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16"/>
       <c r="K16"/>
       <c r="L16"/>
       <c r="M16"/>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17"/>
       <c r="K17"/>
       <c r="L17"/>
       <c r="M17"/>
       <c r="V17"/>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18"/>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19"/>
       <c r="I19"/>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20"/>
     </row>
   </sheetData>
@@ -2896,9 +2899,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4AB1B0E-358B-42C2-9D0A-E02812A76C3C}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H101"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="4" width="26.5703125" customWidth="1"/>
@@ -2907,7 +2909,7 @@
     <col min="8" max="8" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>66</v>
       </c>
@@ -2933,7 +2935,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>73</v>
       </c>
@@ -2943,7 +2945,9 @@
       <c r="C2" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D2" s="6"/>
+      <c r="D2" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="E2" s="6" t="s">
         <v>76</v>
       </c>
@@ -2955,7 +2959,7 @@
       </c>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" hidden="1">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>73</v>
       </c>
@@ -2975,7 +2979,7 @@
       </c>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" hidden="1">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>73</v>
       </c>
@@ -2997,7 +3001,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>73</v>
       </c>
@@ -3017,7 +3021,7 @@
       </c>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:8" hidden="1">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>73</v>
       </c>
@@ -3037,7 +3041,7 @@
       </c>
       <c r="H6" s="6"/>
     </row>
-    <row r="7" spans="1:8" hidden="1">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>73</v>
       </c>
@@ -3057,7 +3061,7 @@
       </c>
       <c r="H7" s="6"/>
     </row>
-    <row r="8" spans="1:8" hidden="1">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>73</v>
       </c>
@@ -3077,7 +3081,7 @@
       </c>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:8" hidden="1">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>73</v>
       </c>
@@ -3097,7 +3101,7 @@
       </c>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:8" hidden="1">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>73</v>
       </c>
@@ -3117,7 +3121,7 @@
       </c>
       <c r="H10" s="6"/>
     </row>
-    <row r="11" spans="1:8" hidden="1">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>73</v>
       </c>
@@ -3137,7 +3141,7 @@
       </c>
       <c r="H11" s="6"/>
     </row>
-    <row r="12" spans="1:8" hidden="1">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>73</v>
       </c>
@@ -3157,7 +3161,7 @@
       </c>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" spans="1:8" hidden="1">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>73</v>
       </c>
@@ -3177,7 +3181,7 @@
       </c>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:8" hidden="1">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>73</v>
       </c>
@@ -3197,7 +3201,7 @@
       </c>
       <c r="H14" s="6"/>
     </row>
-    <row r="15" spans="1:8" hidden="1">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>96</v>
       </c>
@@ -3219,7 +3223,7 @@
       </c>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:8" hidden="1">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>96</v>
       </c>
@@ -3241,7 +3245,7 @@
       </c>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="1:8" hidden="1">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>96</v>
       </c>
@@ -3263,7 +3267,7 @@
       </c>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:8" hidden="1">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>96</v>
       </c>
@@ -3285,7 +3289,7 @@
       </c>
       <c r="H18" s="6"/>
     </row>
-    <row r="19" spans="1:8" hidden="1">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>96</v>
       </c>
@@ -3307,7 +3311,7 @@
       </c>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="1:8" hidden="1">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>96</v>
       </c>
@@ -3329,7 +3333,7 @@
       </c>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:8" hidden="1">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>96</v>
       </c>
@@ -3351,7 +3355,7 @@
       </c>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" spans="1:8" hidden="1">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>96</v>
       </c>
@@ -3373,7 +3377,7 @@
       </c>
       <c r="H22" s="6"/>
     </row>
-    <row r="23" spans="1:8" hidden="1">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>96</v>
       </c>
@@ -3395,7 +3399,7 @@
       </c>
       <c r="H23" s="6"/>
     </row>
-    <row r="24" spans="1:8" hidden="1">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>96</v>
       </c>
@@ -3417,7 +3421,7 @@
       </c>
       <c r="H24" s="6"/>
     </row>
-    <row r="25" spans="1:8" hidden="1">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>96</v>
       </c>
@@ -3439,7 +3443,7 @@
       </c>
       <c r="H25" s="6"/>
     </row>
-    <row r="26" spans="1:8" hidden="1">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>96</v>
       </c>
@@ -3461,7 +3465,7 @@
       </c>
       <c r="H26" s="6"/>
     </row>
-    <row r="27" spans="1:8" hidden="1">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>96</v>
       </c>
@@ -3483,7 +3487,7 @@
       </c>
       <c r="H27" s="6"/>
     </row>
-    <row r="28" spans="1:8" hidden="1">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>96</v>
       </c>
@@ -3505,7 +3509,7 @@
       </c>
       <c r="H28" s="6"/>
     </row>
-    <row r="29" spans="1:8" hidden="1">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>96</v>
       </c>
@@ -3527,7 +3531,7 @@
       </c>
       <c r="H29" s="6"/>
     </row>
-    <row r="30" spans="1:8" hidden="1">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>96</v>
       </c>
@@ -3549,7 +3553,7 @@
       </c>
       <c r="H30" s="6"/>
     </row>
-    <row r="31" spans="1:8" hidden="1">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>96</v>
       </c>
@@ -3571,7 +3575,7 @@
       </c>
       <c r="H31" s="6"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>128</v>
       </c>
@@ -3591,7 +3595,7 @@
       </c>
       <c r="H32" s="6"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>128</v>
       </c>
@@ -3611,7 +3615,7 @@
       </c>
       <c r="H33" s="6"/>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>128</v>
       </c>
@@ -3631,7 +3635,7 @@
       </c>
       <c r="H34" s="6"/>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>128</v>
       </c>
@@ -3651,7 +3655,7 @@
       </c>
       <c r="H35" s="6"/>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>128</v>
       </c>
@@ -3671,7 +3675,7 @@
       </c>
       <c r="H36" s="6"/>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>128</v>
       </c>
@@ -3691,7 +3695,7 @@
       </c>
       <c r="H37" s="6"/>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>128</v>
       </c>
@@ -3711,7 +3715,7 @@
       </c>
       <c r="H38" s="6"/>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>128</v>
       </c>
@@ -3731,7 +3735,7 @@
       </c>
       <c r="H39" s="6"/>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>128</v>
       </c>
@@ -3751,7 +3755,7 @@
       </c>
       <c r="H40" s="6"/>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>128</v>
       </c>
@@ -3771,7 +3775,7 @@
       </c>
       <c r="H41" s="6"/>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>128</v>
       </c>
@@ -3791,7 +3795,7 @@
       </c>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>128</v>
       </c>
@@ -3811,7 +3815,7 @@
       </c>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>128</v>
       </c>
@@ -3831,7 +3835,7 @@
       </c>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>128</v>
       </c>
@@ -3851,7 +3855,7 @@
       </c>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>128</v>
       </c>
@@ -3871,7 +3875,7 @@
       </c>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>128</v>
       </c>
@@ -3891,7 +3895,7 @@
       </c>
       <c r="H47" s="6"/>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>128</v>
       </c>
@@ -3911,7 +3915,7 @@
       </c>
       <c r="H48" s="6"/>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>128</v>
       </c>
@@ -3931,7 +3935,7 @@
       </c>
       <c r="H49" s="6"/>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>128</v>
       </c>
@@ -3951,7 +3955,7 @@
       </c>
       <c r="H50" s="6"/>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>128</v>
       </c>
@@ -3971,7 +3975,7 @@
       </c>
       <c r="H51" s="6"/>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>128</v>
       </c>
@@ -3991,7 +3995,7 @@
       </c>
       <c r="H52" s="6"/>
     </row>
-    <row r="53" spans="1:8" hidden="1">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>162</v>
       </c>
@@ -4011,7 +4015,7 @@
       </c>
       <c r="H53" s="6"/>
     </row>
-    <row r="54" spans="1:8" hidden="1">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>162</v>
       </c>
@@ -4031,7 +4035,7 @@
       </c>
       <c r="H54" s="6"/>
     </row>
-    <row r="55" spans="1:8" hidden="1">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>162</v>
       </c>
@@ -4051,7 +4055,7 @@
       </c>
       <c r="H55" s="6"/>
     </row>
-    <row r="56" spans="1:8" hidden="1">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>162</v>
       </c>
@@ -4071,7 +4075,7 @@
       </c>
       <c r="H56" s="6"/>
     </row>
-    <row r="57" spans="1:8" hidden="1">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>162</v>
       </c>
@@ -4091,7 +4095,7 @@
       </c>
       <c r="H57" s="6"/>
     </row>
-    <row r="58" spans="1:8" hidden="1">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>162</v>
       </c>
@@ -4111,7 +4115,7 @@
       </c>
       <c r="H58" s="6"/>
     </row>
-    <row r="59" spans="1:8" hidden="1">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>162</v>
       </c>
@@ -4131,7 +4135,7 @@
       </c>
       <c r="H59" s="6"/>
     </row>
-    <row r="60" spans="1:8" hidden="1">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>162</v>
       </c>
@@ -4151,7 +4155,7 @@
       </c>
       <c r="H60" s="6"/>
     </row>
-    <row r="61" spans="1:8" hidden="1">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>162</v>
       </c>
@@ -4171,7 +4175,7 @@
       </c>
       <c r="H61" s="6"/>
     </row>
-    <row r="62" spans="1:8" hidden="1">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>162</v>
       </c>
@@ -4191,7 +4195,7 @@
       </c>
       <c r="H62" s="6"/>
     </row>
-    <row r="63" spans="1:8" hidden="1">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>162</v>
       </c>
@@ -4211,7 +4215,7 @@
       </c>
       <c r="H63" s="6"/>
     </row>
-    <row r="64" spans="1:8" hidden="1">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>162</v>
       </c>
@@ -4231,7 +4235,7 @@
       </c>
       <c r="H64" s="6"/>
     </row>
-    <row r="65" spans="1:8" hidden="1">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>192</v>
       </c>
@@ -4251,7 +4255,7 @@
       </c>
       <c r="H65" s="6"/>
     </row>
-    <row r="66" spans="1:8" hidden="1">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>192</v>
       </c>
@@ -4271,7 +4275,7 @@
       </c>
       <c r="H66" s="6"/>
     </row>
-    <row r="67" spans="1:8" hidden="1">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>192</v>
       </c>
@@ -4291,7 +4295,7 @@
       </c>
       <c r="H67" s="6"/>
     </row>
-    <row r="68" spans="1:8" hidden="1">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>192</v>
       </c>
@@ -4311,7 +4315,7 @@
       </c>
       <c r="H68" s="6"/>
     </row>
-    <row r="69" spans="1:8" hidden="1">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>192</v>
       </c>
@@ -4331,7 +4335,7 @@
       </c>
       <c r="H69" s="6"/>
     </row>
-    <row r="70" spans="1:8" hidden="1">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>192</v>
       </c>
@@ -4351,7 +4355,7 @@
       </c>
       <c r="H70" s="6"/>
     </row>
-    <row r="71" spans="1:8" hidden="1">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>192</v>
       </c>
@@ -4371,7 +4375,7 @@
       </c>
       <c r="H71" s="6"/>
     </row>
-    <row r="72" spans="1:8" hidden="1">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>192</v>
       </c>
@@ -4391,7 +4395,7 @@
       </c>
       <c r="H72" s="6"/>
     </row>
-    <row r="73" spans="1:8" hidden="1">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>192</v>
       </c>
@@ -4411,7 +4415,7 @@
       </c>
       <c r="H73" s="6"/>
     </row>
-    <row r="74" spans="1:8" hidden="1">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>192</v>
       </c>
@@ -4431,7 +4435,7 @@
       </c>
       <c r="H74" s="6"/>
     </row>
-    <row r="75" spans="1:8" hidden="1">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>211</v>
       </c>
@@ -4451,7 +4455,7 @@
       </c>
       <c r="H75" s="6"/>
     </row>
-    <row r="76" spans="1:8" hidden="1">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>211</v>
       </c>
@@ -4471,7 +4475,7 @@
       </c>
       <c r="H76" s="6"/>
     </row>
-    <row r="77" spans="1:8" hidden="1">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>211</v>
       </c>
@@ -4491,7 +4495,7 @@
       </c>
       <c r="H77" s="6"/>
     </row>
-    <row r="78" spans="1:8" hidden="1">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>211</v>
       </c>
@@ -4511,7 +4515,7 @@
       </c>
       <c r="H78" s="6"/>
     </row>
-    <row r="79" spans="1:8" hidden="1">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>211</v>
       </c>
@@ -4531,7 +4535,7 @@
       </c>
       <c r="H79" s="6"/>
     </row>
-    <row r="80" spans="1:8" hidden="1">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>211</v>
       </c>
@@ -4551,7 +4555,7 @@
       </c>
       <c r="H80" s="6"/>
     </row>
-    <row r="81" spans="1:8" hidden="1">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>211</v>
       </c>
@@ -4571,7 +4575,7 @@
       </c>
       <c r="H81" s="6"/>
     </row>
-    <row r="82" spans="1:8" hidden="1">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>211</v>
       </c>
@@ -4591,7 +4595,7 @@
       </c>
       <c r="H82" s="6"/>
     </row>
-    <row r="83" spans="1:8" hidden="1">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>211</v>
       </c>
@@ -4611,7 +4615,7 @@
       </c>
       <c r="H83" s="6"/>
     </row>
-    <row r="84" spans="1:8" hidden="1">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>211</v>
       </c>
@@ -4631,7 +4635,7 @@
       </c>
       <c r="H84" s="6"/>
     </row>
-    <row r="85" spans="1:8" hidden="1">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>211</v>
       </c>
@@ -4651,7 +4655,7 @@
       </c>
       <c r="H85" s="6"/>
     </row>
-    <row r="86" spans="1:8" hidden="1">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>211</v>
       </c>
@@ -4671,7 +4675,7 @@
       </c>
       <c r="H86" s="6"/>
     </row>
-    <row r="87" spans="1:8" hidden="1">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>211</v>
       </c>
@@ -4691,7 +4695,7 @@
       </c>
       <c r="H87" s="6"/>
     </row>
-    <row r="88" spans="1:8" hidden="1">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>211</v>
       </c>
@@ -4711,7 +4715,7 @@
       </c>
       <c r="H88" s="6"/>
     </row>
-    <row r="89" spans="1:8" hidden="1">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>211</v>
       </c>
@@ -4731,7 +4735,7 @@
       </c>
       <c r="H89" s="6"/>
     </row>
-    <row r="90" spans="1:8" hidden="1">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>211</v>
       </c>
@@ -4751,7 +4755,7 @@
       </c>
       <c r="H90" s="6"/>
     </row>
-    <row r="91" spans="1:8" hidden="1">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>211</v>
       </c>
@@ -4771,7 +4775,7 @@
       </c>
       <c r="H91" s="6"/>
     </row>
-    <row r="92" spans="1:8" hidden="1">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>211</v>
       </c>
@@ -4791,7 +4795,7 @@
       </c>
       <c r="H92" s="6"/>
     </row>
-    <row r="93" spans="1:8" hidden="1">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>211</v>
       </c>
@@ -4811,7 +4815,7 @@
       </c>
       <c r="H93" s="6"/>
     </row>
-    <row r="94" spans="1:8" hidden="1">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>211</v>
       </c>
@@ -4831,7 +4835,7 @@
       </c>
       <c r="H94" s="6"/>
     </row>
-    <row r="95" spans="1:8" hidden="1">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>211</v>
       </c>
@@ -4851,7 +4855,7 @@
       </c>
       <c r="H95" s="6"/>
     </row>
-    <row r="96" spans="1:8" hidden="1">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>211</v>
       </c>
@@ -4871,7 +4875,7 @@
       </c>
       <c r="H96" s="6"/>
     </row>
-    <row r="97" spans="1:8" hidden="1">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>211</v>
       </c>
@@ -4891,7 +4895,7 @@
       </c>
       <c r="H97" s="6"/>
     </row>
-    <row r="98" spans="1:8" hidden="1">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>211</v>
       </c>
@@ -4911,7 +4915,7 @@
       </c>
       <c r="H98" s="6"/>
     </row>
-    <row r="99" spans="1:8" hidden="1">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>211</v>
       </c>
@@ -4931,7 +4935,7 @@
       </c>
       <c r="H99" s="6"/>
     </row>
-    <row r="100" spans="1:8" hidden="1">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>211</v>
       </c>
@@ -4951,7 +4955,7 @@
       </c>
       <c r="H100" s="6"/>
     </row>
-    <row r="101" spans="1:8" hidden="1">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>211</v>
       </c>
@@ -4972,13 +4976,7 @@
       <c r="H101" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I101" xr:uid="{A4AB1B0E-358B-42C2-9D0A-E02812A76C3C}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Дальний Восток"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I101" xr:uid="{A4AB1B0E-358B-42C2-9D0A-E02812A76C3C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4986,7 +4984,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D34489A3-A8B0-4D6F-A6E8-B4FAFCF5D4F6}">
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -4997,7 +4995,7 @@
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>66</v>
       </c>
@@ -5020,7 +5018,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>73</v>
       </c>
@@ -5041,7 +5039,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>73</v>
       </c>
@@ -5062,7 +5060,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>73</v>
       </c>
@@ -5083,7 +5081,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>73</v>
       </c>
@@ -5104,7 +5102,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>73</v>
       </c>
@@ -5125,7 +5123,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>162</v>
       </c>
@@ -5148,7 +5146,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>162</v>
       </c>
@@ -5169,7 +5167,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>162</v>
       </c>
@@ -5190,7 +5188,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>162</v>
       </c>
@@ -5214,7 +5212,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>162</v>
       </c>
@@ -5238,7 +5236,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>162</v>
       </c>
@@ -5262,7 +5260,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>162</v>
       </c>
@@ -5283,7 +5281,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>162</v>
       </c>
@@ -5304,7 +5302,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>162</v>
       </c>
@@ -5325,7 +5323,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>192</v>
       </c>
@@ -5346,7 +5344,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>192</v>
       </c>
@@ -5367,7 +5365,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>192</v>
       </c>
@@ -5388,7 +5386,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>192</v>
       </c>
@@ -5409,7 +5407,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>192</v>
       </c>
@@ -5430,7 +5428,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>192</v>
       </c>
@@ -5451,7 +5449,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>192</v>
       </c>
@@ -5472,7 +5470,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>192</v>
       </c>
@@ -5493,7 +5491,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -5502,7 +5500,7 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -5511,7 +5509,7 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -5520,7 +5518,7 @@
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -5529,7 +5527,7 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -5538,7 +5536,7 @@
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -5555,7 +5553,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F033FB-4DB8-4067-A8C0-4DACAF03F6E6}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>